<commit_message>
automation project code commited
</commit_message>
<xml_diff>
--- a/src/test/resources/Testdata/testdata.xlsx
+++ b/src/test/resources/Testdata/testdata.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Selenium Course\MySeleniumSessions\FrameWorkPractice27012026\selenium-framework\src\test\resources\Testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\BusinessnextPortal\src\test\resources\Testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>HDFC Cloud Migration - Track 2</t>
   </si>
@@ -74,7 +74,10 @@
     <t>TC_02</t>
   </si>
   <si>
-    <t>dfgbndfgbfd</t>
+    <t>Applies_To_value</t>
+  </si>
+  <si>
+    <t>Public IP2</t>
   </si>
   <si>
     <t>Fail</t>
@@ -399,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="28.42578125"/>
@@ -408,13 +411,14 @@
     <col min="5" max="5" bestFit="true" customWidth="true" width="17.85546875"/>
     <col min="6" max="6" bestFit="true" customWidth="true" width="11.5703125"/>
     <col min="7" max="7" bestFit="true" customWidth="true" width="17.85546875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="11.42578125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="12.140625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="11.5703125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="16.85546875"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="11.42578125"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="12.85546875"/>
+    <col min="15" max="15" bestFit="true" customWidth="true" width="12.140625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="11.5703125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s" s="0">
         <v>11</v>
       </c>
@@ -437,10 +441,13 @@
         <v>9</v>
       </c>
       <c r="H1" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="I1" t="s" s="0">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
         <v>12</v>
       </c>
@@ -463,10 +470,13 @@
         <v>10</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s" s="0">
         <v>15</v>
       </c>
@@ -477,7 +487,7 @@
         <v>13</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>6</v>
@@ -490,6 +500,9 @@
       </c>
       <c r="H3" t="s" s="0">
         <v>17</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>